<commit_message>
work log excel update
</commit_message>
<xml_diff>
--- a/requirements/Hexapod_Anforderung_250916.xlsx
+++ b/requirements/Hexapod_Anforderung_250916.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\linus\OneDrive\Desktop\Hexapod\requirements\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{DA68305B-6858-4749-8037-1CD3CD00DF61}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{CE1BA0F9-481F-4764-87D9-0BC9670BC0E5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="38280" yWindow="-630" windowWidth="38640" windowHeight="21120" xr2:uid="{4078619B-BBF7-437A-BD9C-8FC6100B879D}"/>
   </bookViews>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="56" uniqueCount="30">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="54" uniqueCount="29">
   <si>
     <t>Funktionale Anforderungen</t>
   </si>
@@ -54,9 +54,6 @@
   </si>
   <si>
     <t>Vom Kunden abgenommen</t>
-  </si>
-  <si>
-    <t>Das Hexapod hat eine IMU.</t>
   </si>
   <si>
     <t>Das Hexapod hat einen Indikator, der anzeigt, wenn die Kamera 
@@ -67,9 +64,6 @@
 und so wenig Klebstoff wie möglich verwendet werden.</t>
   </si>
   <si>
-    <t>Das Hexapod muss im unbewaffneten Zustand programmierbar sein.</t>
-  </si>
-  <si>
     <t>Das Hexapod muss auch im komplett zusammengebauten Zustand 
 noch programmierbar sein.</t>
   </si>
@@ -77,21 +71,12 @@
     <t>Das Hexapod darf 80°C nicht überschreiten.</t>
   </si>
   <si>
-    <t>Das Hexapod kann mit 6V-8,4V gespeist werden.</t>
-  </si>
-  <si>
     <t>Der Akku kann konstant überwacht und per Software ausgeschalten werden können.</t>
   </si>
   <si>
     <t>Die Leistungsaufnahme kann maximal 850W betragen.</t>
   </si>
   <si>
-    <t>Es kann einen Anschluss für Erweiterungen haben (I2C, 5V, GND, 2x GPIO).</t>
-  </si>
-  <si>
-    <t>Es kann einen Überstromschutz und eine Überspannungsschutzschaltung für den Akku haben.</t>
-  </si>
-  <si>
     <t>Das Hexapod kann per Fernbedienung gesteuert werden.</t>
   </si>
   <si>
@@ -107,9 +92,6 @@
     <t>Jedes Bein kann einzeln entfernt werden.</t>
   </si>
   <si>
-    <t>Das Hexapod muss in jeder situation unbewaffnet werden können</t>
-  </si>
-  <si>
     <t>Die Füße sind austauschbar sein.</t>
   </si>
   <si>
@@ -125,10 +107,25 @@
     <t>Das Hexapod ist mit ausgestreckten Beinen unter einem Meter lang.</t>
   </si>
   <si>
-    <t>Das Hexapod hat Anschlüsse für Erweiterungen.</t>
-  </si>
-  <si>
     <t>Das Hexapod wiegt unter 3kg.</t>
+  </si>
+  <si>
+    <t>Das Hexapod muss im "unarmed" Zustand programmierbar sein.</t>
+  </si>
+  <si>
+    <t>Das Hexapod muss in jeder situation in den Zustand "unarmed" gebracht werden können</t>
+  </si>
+  <si>
+    <t>Das Hexapod wird mit 6V-8,4V gespeist werden.</t>
+  </si>
+  <si>
+    <t>Das Hexapod hat eine IMU (Internal Mesurment Unit, kann beschleunigung und rotation in allen Achsen messen).</t>
+  </si>
+  <si>
+    <t>Es hat einen Überstromschutz und eine Unterspannungsschutz für den Akku.</t>
+  </si>
+  <si>
+    <t>das Hexapod hat einen Anschluss für Erweiterungen mit folgenden Anschlüsse: I2C, 5V, GND, 2x GPIO</t>
   </si>
 </sst>
 </file>
@@ -196,8 +193,8 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="3" xr:uid="{8CE789CB-2DE6-4E0D-90E5-F8D531C1A5BA}" name="Tabelle1" displayName="Tabelle1" ref="B4:D22" totalsRowShown="0">
-  <autoFilter ref="B4:D22" xr:uid="{8CE789CB-2DE6-4E0D-90E5-F8D531C1A5BA}"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="3" xr:uid="{8CE789CB-2DE6-4E0D-90E5-F8D531C1A5BA}" name="Tabelle1" displayName="Tabelle1" ref="B4:D16" totalsRowShown="0">
+  <autoFilter ref="B4:D16" xr:uid="{8CE789CB-2DE6-4E0D-90E5-F8D531C1A5BA}"/>
   <tableColumns count="3">
     <tableColumn id="1" xr3:uid="{9C7CB87B-1858-4EA7-A982-57FB1C283CAB}" name="#"/>
     <tableColumn id="2" xr3:uid="{628C5DE5-E97D-4FA3-9335-A0236E76BEAF}" name="Anforderung "/>
@@ -208,8 +205,8 @@
 </file>
 
 <file path=xl/tables/table2.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="4" xr:uid="{8F15C0C2-9758-4749-8205-DD54A72C72C1}" name="Tabelle4" displayName="Tabelle4" ref="F4:H10" totalsRowShown="0">
-  <autoFilter ref="F4:H10" xr:uid="{8F15C0C2-9758-4749-8205-DD54A72C72C1}"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="4" xr:uid="{8F15C0C2-9758-4749-8205-DD54A72C72C1}" name="Tabelle4" displayName="Tabelle4" ref="F4:H16" totalsRowShown="0">
+  <autoFilter ref="F4:H16" xr:uid="{8F15C0C2-9758-4749-8205-DD54A72C72C1}"/>
   <tableColumns count="3">
     <tableColumn id="1" xr3:uid="{1A4D7D2C-212C-4CD4-A15C-D97AF066D995}" name="#"/>
     <tableColumn id="2" xr3:uid="{25A58F6B-DF12-49E9-B658-3DA940401B0E}" name="Anforderung "/>
@@ -536,7 +533,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{FE7D0DD2-8A3B-41E7-A9D4-526B964DFBAE}">
-  <dimension ref="B2:H22"/>
+  <dimension ref="B2:H16"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="3" max="3" width="61.28515625" customWidth="1"/>
@@ -578,7 +575,7 @@
         <v>1</v>
       </c>
       <c r="C5" t="s">
-        <v>17</v>
+        <v>12</v>
       </c>
       <c r="D5" t="s">
         <v>5</v>
@@ -587,7 +584,7 @@
         <v>1</v>
       </c>
       <c r="G5" t="s">
-        <v>25</v>
+        <v>19</v>
       </c>
       <c r="H5" t="s">
         <v>5</v>
@@ -598,7 +595,7 @@
         <v>2</v>
       </c>
       <c r="C6" t="s">
-        <v>18</v>
+        <v>13</v>
       </c>
       <c r="D6" t="s">
         <v>5</v>
@@ -607,7 +604,7 @@
         <v>2</v>
       </c>
       <c r="G6" t="s">
-        <v>27</v>
+        <v>21</v>
       </c>
       <c r="H6" t="s">
         <v>5</v>
@@ -618,19 +615,13 @@
         <v>3</v>
       </c>
       <c r="C7" t="s">
-        <v>12</v>
+        <v>25</v>
       </c>
       <c r="D7" t="s">
         <v>5</v>
       </c>
       <c r="F7">
         <v>3</v>
-      </c>
-      <c r="G7" t="s">
-        <v>28</v>
-      </c>
-      <c r="H7" t="s">
-        <v>5</v>
       </c>
     </row>
     <row r="8" spans="2:8" x14ac:dyDescent="0.25">
@@ -638,7 +629,7 @@
         <v>4</v>
       </c>
       <c r="C8" t="s">
-        <v>19</v>
+        <v>14</v>
       </c>
       <c r="D8" t="s">
         <v>5</v>
@@ -647,13 +638,13 @@
         <v>4</v>
       </c>
       <c r="G8" t="s">
-        <v>26</v>
+        <v>20</v>
       </c>
       <c r="H8" t="s">
         <v>5</v>
       </c>
     </row>
-    <row r="9" spans="2:8" x14ac:dyDescent="0.25">
+    <row r="9" spans="2:8" ht="30" x14ac:dyDescent="0.25">
       <c r="B9">
         <v>5</v>
       </c>
@@ -666,8 +657,8 @@
       <c r="F9">
         <v>5</v>
       </c>
-      <c r="G9" t="s">
-        <v>29</v>
+      <c r="G9" s="2" t="s">
+        <v>7</v>
       </c>
       <c r="H9" t="s">
         <v>5</v>
@@ -678,7 +669,7 @@
         <v>6</v>
       </c>
       <c r="C10" s="2" t="s">
-        <v>7</v>
+        <v>24</v>
       </c>
       <c r="D10" t="s">
         <v>5</v>
@@ -687,53 +678,89 @@
         <v>6</v>
       </c>
       <c r="G10" s="2" t="s">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="H10" t="s">
         <v>5</v>
       </c>
     </row>
-    <row r="11" spans="2:8" x14ac:dyDescent="0.25">
+    <row r="11" spans="2:8" ht="30" x14ac:dyDescent="0.25">
       <c r="B11">
         <v>7</v>
       </c>
-      <c r="C11" t="s">
-        <v>20</v>
+      <c r="C11" s="2" t="s">
+        <v>10</v>
       </c>
       <c r="D11" t="s">
         <v>5</v>
       </c>
-    </row>
-    <row r="12" spans="2:8" x14ac:dyDescent="0.25">
+      <c r="F11">
+        <v>7</v>
+      </c>
+      <c r="G11" s="2" t="s">
+        <v>23</v>
+      </c>
+      <c r="H11" t="s">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="12" spans="2:8" ht="30" x14ac:dyDescent="0.25">
       <c r="B12">
         <v>8</v>
       </c>
-      <c r="C12" t="s">
-        <v>21</v>
+      <c r="C12" s="2" t="s">
+        <v>11</v>
       </c>
       <c r="D12" t="s">
         <v>5</v>
       </c>
-    </row>
-    <row r="13" spans="2:8" x14ac:dyDescent="0.25">
+      <c r="F12">
+        <v>8</v>
+      </c>
+      <c r="G12" s="2" t="s">
+        <v>26</v>
+      </c>
+      <c r="H12" t="s">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="13" spans="2:8" ht="30" x14ac:dyDescent="0.25">
       <c r="B13">
         <v>9</v>
       </c>
       <c r="C13" s="2" t="s">
-        <v>22</v>
+        <v>28</v>
       </c>
       <c r="D13" t="s">
         <v>5</v>
       </c>
-    </row>
-    <row r="14" spans="2:8" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="F13">
+        <v>9</v>
+      </c>
+      <c r="G13" t="s">
+        <v>15</v>
+      </c>
+      <c r="H13" t="s">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="14" spans="2:8" ht="29.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B14">
         <v>10</v>
       </c>
       <c r="C14" s="2" t="s">
-        <v>9</v>
+        <v>27</v>
       </c>
       <c r="D14" t="s">
+        <v>5</v>
+      </c>
+      <c r="F14">
+        <v>10</v>
+      </c>
+      <c r="G14" t="s">
+        <v>16</v>
+      </c>
+      <c r="H14" t="s">
         <v>5</v>
       </c>
     </row>
@@ -742,86 +769,38 @@
         <v>11</v>
       </c>
       <c r="C15" s="2" t="s">
-        <v>10</v>
+        <v>18</v>
       </c>
       <c r="D15" t="s">
         <v>5</v>
       </c>
-    </row>
-    <row r="16" spans="2:8" ht="30" x14ac:dyDescent="0.25">
+      <c r="F15">
+        <v>11</v>
+      </c>
+      <c r="G15" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="H15" t="s">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="16" spans="2:8" x14ac:dyDescent="0.25">
       <c r="B16">
+        <v>11</v>
+      </c>
+      <c r="C16" t="s">
+        <v>22</v>
+      </c>
+      <c r="D16" t="s">
+        <v>5</v>
+      </c>
+      <c r="F16">
         <v>12</v>
       </c>
-      <c r="C16" s="2" t="s">
-        <v>13</v>
-      </c>
-      <c r="D16" t="s">
-        <v>5</v>
-      </c>
-    </row>
-    <row r="17" spans="2:4" x14ac:dyDescent="0.25">
-      <c r="B17">
-        <v>13</v>
-      </c>
-      <c r="C17" s="2" t="s">
-        <v>11</v>
-      </c>
-      <c r="D17" t="s">
-        <v>5</v>
-      </c>
-    </row>
-    <row r="18" spans="2:4" x14ac:dyDescent="0.25">
-      <c r="B18">
-        <v>14</v>
-      </c>
-      <c r="C18" s="2" t="s">
-        <v>14</v>
-      </c>
-      <c r="D18" t="s">
-        <v>5</v>
-      </c>
-    </row>
-    <row r="19" spans="2:4" ht="30" x14ac:dyDescent="0.25">
-      <c r="B19">
-        <v>15</v>
-      </c>
-      <c r="C19" s="2" t="s">
-        <v>15</v>
-      </c>
-      <c r="D19" t="s">
-        <v>5</v>
-      </c>
-    </row>
-    <row r="20" spans="2:4" ht="30" x14ac:dyDescent="0.25">
-      <c r="B20">
-        <v>16</v>
-      </c>
-      <c r="C20" s="2" t="s">
-        <v>16</v>
-      </c>
-      <c r="D20" t="s">
-        <v>5</v>
-      </c>
-    </row>
-    <row r="21" spans="2:4" x14ac:dyDescent="0.25">
-      <c r="B21">
+      <c r="G16" s="2" t="s">
         <v>17</v>
       </c>
-      <c r="C21" s="2" t="s">
-        <v>23</v>
-      </c>
-      <c r="D21" t="s">
-        <v>5</v>
-      </c>
-    </row>
-    <row r="22" spans="2:4" x14ac:dyDescent="0.25">
-      <c r="B22">
-        <v>18</v>
-      </c>
-      <c r="C22" s="2" t="s">
-        <v>24</v>
-      </c>
-      <c r="D22" t="s">
+      <c r="H16" t="s">
         <v>5</v>
       </c>
     </row>
@@ -844,6 +823,14 @@
 </file>
 
 <file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement>
+    <_activity xmlns="5f1a80e9-d6bc-4031-b10f-d21f31a30176" xsi:nil="true"/>
+  </documentManagement>
+</p:properties>
+</file>
+
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Dokument" ma:contentTypeID="0x0101005A8D12E036A38A4C82FA7B9385EF06A9" ma:contentTypeVersion="15" ma:contentTypeDescription="Ein neues Dokument erstellen." ma:contentTypeScope="" ma:versionID="5847bb9604bf2beda18d4f7cd4b8a0bc">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns3="5f1a80e9-d6bc-4031-b10f-d21f31a30176" xmlns:ns4="dce9bcdd-9eea-4ca5-a49c-ebeb07b55999" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="02ca0f69bb2fee6ab7e7537675a9b63c" ns3:_="" ns4:_="">
     <xsd:import namespace="5f1a80e9-d6bc-4031-b10f-d21f31a30176"/>
@@ -1076,14 +1063,6 @@
 </ct:contentTypeSchema>
 </file>
 
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement>
-    <_activity xmlns="5f1a80e9-d6bc-4031-b10f-d21f31a30176" xsi:nil="true"/>
-  </documentManagement>
-</p:properties>
-</file>
-
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{C50BBE33-4FF4-4BA4-8155-4BCE83228CBA}">
   <ds:schemaRefs>
@@ -1093,6 +1072,23 @@
 </file>
 
 <file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{7613F5EA-D984-4CF2-A0F8-E6A2B088D052}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="5f1a80e9-d6bc-4031-b10f-d21f31a30176"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
+    <ds:schemaRef ds:uri="http://www.w3.org/XML/1998/namespace"/>
+    <ds:schemaRef ds:uri="dce9bcdd-9eea-4ca5-a49c-ebeb07b55999"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/dcmitype/"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
+</file>
+
+<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{C95935A0-F985-4FFC-9287-686DBD7B5494}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
@@ -1109,21 +1105,4 @@
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/internal/obd"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
-</file>
-
-<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{7613F5EA-D984-4CF2-A0F8-E6A2B088D052}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="5f1a80e9-d6bc-4031-b10f-d21f31a30176"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
-    <ds:schemaRef ds:uri="http://www.w3.org/XML/1998/namespace"/>
-    <ds:schemaRef ds:uri="dce9bcdd-9eea-4ca5-a49c-ebeb07b55999"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/dcmitype/"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
 </file>
</xml_diff>

<commit_message>
Doku and cleaning up
</commit_message>
<xml_diff>
--- a/requirements/Hexapod_Anforderung_250916.xlsx
+++ b/requirements/Hexapod_Anforderung_250916.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29127"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29426"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\linus\OneDrive\Desktop\Hexapod\requirements\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\linus\Desktop\ETH\Hexapod\requirements\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{CE1BA0F9-481F-4764-87D9-0BC9670BC0E5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7E98B480-EE02-4C07-BA89-5EE1920219B8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="38280" yWindow="-630" windowWidth="38640" windowHeight="21120" xr2:uid="{4078619B-BBF7-437A-BD9C-8FC6100B879D}"/>
+    <workbookView xWindow="-98" yWindow="-98" windowWidth="23236" windowHeight="13875" xr2:uid="{4078619B-BBF7-437A-BD9C-8FC6100B879D}"/>
   </bookViews>
   <sheets>
     <sheet name="Tabelle1" sheetId="1" r:id="rId1"/>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="54" uniqueCount="29">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="108" uniqueCount="41">
   <si>
     <t>Funktionale Anforderungen</t>
   </si>
@@ -126,6 +126,46 @@
   </si>
   <si>
     <t>das Hexapod hat einen Anschluss für Erweiterungen mit folgenden Anschlüsse: I2C, 5V, GND, 2x GPIO</t>
+  </si>
+  <si>
+    <t>Funktionale Anforderungen Test</t>
+  </si>
+  <si>
+    <t>Nichtfunktionale Anforderungen Test</t>
+  </si>
+  <si>
+    <t>Erreicht</t>
+  </si>
+  <si>
+    <t>Erreicht (5.8V-8.4V)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Erreicht (I2C, 5V 2x GPIO, 3.3V, 
+5.8-8.4V, ADC, SPI)
+</t>
+  </si>
+  <si>
+    <t>Erreicht (PS5 Controller)</t>
+  </si>
+  <si>
+    <t>Nicht Erreicht (3.315Kg)</t>
+  </si>
+  <si>
+    <t>Erreicht (PETG)</t>
+  </si>
+  <si>
+    <t>Erreicht (94.53cm)</t>
+  </si>
+  <si>
+    <t>Erreicht (Alles aussert 2 Bauteile sind 
+verschraubt)</t>
+  </si>
+  <si>
+    <t>Erreicht (max temp = 65° (Raspberry pi 5 
+maximale core tempereatur))</t>
+  </si>
+  <si>
+    <t>Noch nicht Erreicht</t>
   </si>
 </sst>
 </file>
@@ -149,12 +189,30 @@
       <scheme val="minor"/>
     </font>
   </fonts>
-  <fills count="2">
+  <fills count="5">
     <fill>
       <patternFill patternType="none"/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="5"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="9"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFF0000"/>
+        <bgColor indexed="64"/>
+      </patternFill>
     </fill>
   </fills>
   <borders count="1">
@@ -169,15 +227,22 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="3">
+  <cellXfs count="8">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1"/>
   </cellXfs>
   <cellStyles count="1">
-    <cellStyle name="Standard" xfId="0" builtinId="0"/>
+    <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
   <dxfs count="0"/>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
@@ -205,8 +270,8 @@
 </file>
 
 <file path=xl/tables/table2.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="4" xr:uid="{8F15C0C2-9758-4749-8205-DD54A72C72C1}" name="Tabelle4" displayName="Tabelle4" ref="F4:H16" totalsRowShown="0">
-  <autoFilter ref="F4:H16" xr:uid="{8F15C0C2-9758-4749-8205-DD54A72C72C1}"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="4" xr:uid="{8F15C0C2-9758-4749-8205-DD54A72C72C1}" name="Tabelle4" displayName="Tabelle4" ref="F4:H15" totalsRowShown="0">
+  <autoFilter ref="F4:H15" xr:uid="{8F15C0C2-9758-4749-8205-DD54A72C72C1}"/>
   <tableColumns count="3">
     <tableColumn id="1" xr3:uid="{1A4D7D2C-212C-4CD4-A15C-D97AF066D995}" name="#"/>
     <tableColumn id="2" xr3:uid="{25A58F6B-DF12-49E9-B658-3DA940401B0E}" name="Anforderung "/>
@@ -216,8 +281,32 @@
 </table>
 </file>
 
+<file path=xl/tables/table3.xml><?xml version="1.0" encoding="utf-8"?>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{2E97DB2C-4CF8-4078-81EF-0FE330324823}" name="Tabelle12" displayName="Tabelle12" ref="B22:D34" totalsRowShown="0">
+  <autoFilter ref="B22:D34" xr:uid="{2E97DB2C-4CF8-4078-81EF-0FE330324823}"/>
+  <tableColumns count="3">
+    <tableColumn id="1" xr3:uid="{BFF90018-1749-4F2C-A01C-712D17FD6C59}" name="#"/>
+    <tableColumn id="2" xr3:uid="{D4B512FB-3AB5-4CDD-8DAB-87E0052BCF7F}" name="Anforderung "/>
+    <tableColumn id="3" xr3:uid="{0DC65304-6390-4943-82F4-9CF4774E947E}" name="Status"/>
+  </tableColumns>
+  <tableStyleInfo name="TableStyleMedium5" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
+</table>
+</file>
+
+<file path=xl/tables/table4.xml><?xml version="1.0" encoding="utf-8"?>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="2" xr:uid="{6A6065B8-E143-41C6-8E02-8903CA03623B}" name="Tabelle43" displayName="Tabelle43" ref="F22:H34" totalsRowShown="0">
+  <autoFilter ref="F22:H34" xr:uid="{6A6065B8-E143-41C6-8E02-8903CA03623B}"/>
+  <tableColumns count="3">
+    <tableColumn id="1" xr3:uid="{723A0041-FE8A-491C-AC63-E0946CD5210B}" name="#"/>
+    <tableColumn id="2" xr3:uid="{698092AB-1765-4F95-930E-C063E03C89CB}" name="Anforderung "/>
+    <tableColumn id="3" xr3:uid="{CC59DB8E-318B-4FA9-BDB1-74C3CA05A692}" name="Status"/>
+  </tableColumns>
+  <tableStyleInfo name="TableStyleMedium5" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
+</table>
+</file>
+
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
-<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office">
+<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme">
   <a:themeElements>
     <a:clrScheme name="Office">
       <a:dk1>
@@ -533,16 +622,16 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{FE7D0DD2-8A3B-41E7-A9D4-526B964DFBAE}">
-  <dimension ref="B2:H16"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <dimension ref="B2:H34"/>
+  <sheetFormatPr defaultColWidth="10.6640625" defaultRowHeight="14.25" x14ac:dyDescent="0.45"/>
   <cols>
-    <col min="3" max="3" width="61.28515625" customWidth="1"/>
-    <col min="4" max="4" width="26.5703125" customWidth="1"/>
-    <col min="7" max="7" width="61.28515625" customWidth="1"/>
-    <col min="8" max="8" width="33.140625" customWidth="1"/>
+    <col min="3" max="3" width="61.265625" customWidth="1"/>
+    <col min="4" max="4" width="26.59765625" customWidth="1"/>
+    <col min="7" max="7" width="61.265625" customWidth="1"/>
+    <col min="8" max="8" width="33.1328125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="2" spans="2:8" ht="31.5" x14ac:dyDescent="0.5">
+    <row r="2" spans="2:8" ht="31.9" x14ac:dyDescent="1">
       <c r="B2" s="1" t="s">
         <v>0</v>
       </c>
@@ -550,7 +639,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="4" spans="2:8" x14ac:dyDescent="0.25">
+    <row r="4" spans="2:8" x14ac:dyDescent="0.45">
       <c r="B4" t="s">
         <v>1</v>
       </c>
@@ -570,7 +659,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="5" spans="2:8" x14ac:dyDescent="0.25">
+    <row r="5" spans="2:8" x14ac:dyDescent="0.45">
       <c r="B5">
         <v>1</v>
       </c>
@@ -590,7 +679,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="6" spans="2:8" x14ac:dyDescent="0.25">
+    <row r="6" spans="2:8" x14ac:dyDescent="0.45">
       <c r="B6">
         <v>2</v>
       </c>
@@ -610,7 +699,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="7" spans="2:8" x14ac:dyDescent="0.25">
+    <row r="7" spans="2:8" x14ac:dyDescent="0.45">
       <c r="B7">
         <v>3</v>
       </c>
@@ -623,8 +712,14 @@
       <c r="F7">
         <v>3</v>
       </c>
-    </row>
-    <row r="8" spans="2:8" x14ac:dyDescent="0.25">
+      <c r="G7" t="s">
+        <v>20</v>
+      </c>
+      <c r="H7" t="s">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="8" spans="2:8" ht="28.5" x14ac:dyDescent="0.45">
       <c r="B8">
         <v>4</v>
       </c>
@@ -637,14 +732,14 @@
       <c r="F8">
         <v>4</v>
       </c>
-      <c r="G8" t="s">
-        <v>20</v>
+      <c r="G8" s="2" t="s">
+        <v>7</v>
       </c>
       <c r="H8" t="s">
         <v>5</v>
       </c>
     </row>
-    <row r="9" spans="2:8" ht="30" x14ac:dyDescent="0.25">
+    <row r="9" spans="2:8" ht="28.5" x14ac:dyDescent="0.45">
       <c r="B9">
         <v>5</v>
       </c>
@@ -658,13 +753,13 @@
         <v>5</v>
       </c>
       <c r="G9" s="2" t="s">
-        <v>7</v>
+        <v>9</v>
       </c>
       <c r="H9" t="s">
         <v>5</v>
       </c>
     </row>
-    <row r="10" spans="2:8" ht="30" x14ac:dyDescent="0.25">
+    <row r="10" spans="2:8" ht="28.5" x14ac:dyDescent="0.45">
       <c r="B10">
         <v>6</v>
       </c>
@@ -678,13 +773,13 @@
         <v>6</v>
       </c>
       <c r="G10" s="2" t="s">
-        <v>9</v>
+        <v>23</v>
       </c>
       <c r="H10" t="s">
         <v>5</v>
       </c>
     </row>
-    <row r="11" spans="2:8" ht="30" x14ac:dyDescent="0.25">
+    <row r="11" spans="2:8" ht="28.5" x14ac:dyDescent="0.45">
       <c r="B11">
         <v>7</v>
       </c>
@@ -698,13 +793,13 @@
         <v>7</v>
       </c>
       <c r="G11" s="2" t="s">
-        <v>23</v>
+        <v>26</v>
       </c>
       <c r="H11" t="s">
         <v>5</v>
       </c>
     </row>
-    <row r="12" spans="2:8" ht="30" x14ac:dyDescent="0.25">
+    <row r="12" spans="2:8" x14ac:dyDescent="0.45">
       <c r="B12">
         <v>8</v>
       </c>
@@ -717,14 +812,14 @@
       <c r="F12">
         <v>8</v>
       </c>
-      <c r="G12" s="2" t="s">
-        <v>26</v>
+      <c r="G12" t="s">
+        <v>15</v>
       </c>
       <c r="H12" t="s">
         <v>5</v>
       </c>
     </row>
-    <row r="13" spans="2:8" ht="30" x14ac:dyDescent="0.25">
+    <row r="13" spans="2:8" ht="28.5" x14ac:dyDescent="0.45">
       <c r="B13">
         <v>9</v>
       </c>
@@ -738,13 +833,13 @@
         <v>9</v>
       </c>
       <c r="G13" t="s">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="H13" t="s">
         <v>5</v>
       </c>
     </row>
-    <row r="14" spans="2:8" ht="29.25" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="14" spans="2:8" ht="29.25" customHeight="1" x14ac:dyDescent="0.45">
       <c r="B14">
         <v>10</v>
       </c>
@@ -757,14 +852,14 @@
       <c r="F14">
         <v>10</v>
       </c>
-      <c r="G14" t="s">
-        <v>16</v>
+      <c r="G14" s="2" t="s">
+        <v>8</v>
       </c>
       <c r="H14" t="s">
         <v>5</v>
       </c>
     </row>
-    <row r="15" spans="2:8" ht="30" x14ac:dyDescent="0.25">
+    <row r="15" spans="2:8" x14ac:dyDescent="0.45">
       <c r="B15">
         <v>11</v>
       </c>
@@ -778,13 +873,13 @@
         <v>11</v>
       </c>
       <c r="G15" s="2" t="s">
-        <v>8</v>
+        <v>17</v>
       </c>
       <c r="H15" t="s">
         <v>5</v>
       </c>
     </row>
-    <row r="16" spans="2:8" x14ac:dyDescent="0.25">
+    <row r="16" spans="2:8" x14ac:dyDescent="0.45">
       <c r="B16">
         <v>11</v>
       </c>
@@ -794,43 +889,284 @@
       <c r="D16" t="s">
         <v>5</v>
       </c>
-      <c r="F16">
+    </row>
+    <row r="18" spans="2:8" x14ac:dyDescent="0.45">
+      <c r="D18" s="7"/>
+    </row>
+    <row r="19" spans="2:8" x14ac:dyDescent="0.45">
+      <c r="G19" s="7"/>
+    </row>
+    <row r="20" spans="2:8" ht="31.9" x14ac:dyDescent="1">
+      <c r="B20" s="1" t="s">
+        <v>29</v>
+      </c>
+      <c r="F20" s="1" t="s">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="22" spans="2:8" x14ac:dyDescent="0.45">
+      <c r="B22" t="s">
+        <v>1</v>
+      </c>
+      <c r="C22" t="s">
+        <v>2</v>
+      </c>
+      <c r="D22" t="s">
+        <v>3</v>
+      </c>
+      <c r="F22" t="s">
+        <v>1</v>
+      </c>
+      <c r="G22" t="s">
+        <v>2</v>
+      </c>
+      <c r="H22" t="s">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="23" spans="2:8" x14ac:dyDescent="0.45">
+      <c r="B23">
+        <v>1</v>
+      </c>
+      <c r="C23" t="s">
         <v>12</v>
       </c>
-      <c r="G16" s="2" t="s">
+      <c r="D23" s="3" t="s">
+        <v>40</v>
+      </c>
+      <c r="F23">
+        <v>1</v>
+      </c>
+      <c r="G23" t="s">
+        <v>19</v>
+      </c>
+      <c r="H23" s="4" t="s">
+        <v>36</v>
+      </c>
+    </row>
+    <row r="24" spans="2:8" x14ac:dyDescent="0.45">
+      <c r="B24">
+        <v>2</v>
+      </c>
+      <c r="C24" t="s">
+        <v>13</v>
+      </c>
+      <c r="D24" s="4" t="s">
+        <v>31</v>
+      </c>
+      <c r="F24">
+        <v>2</v>
+      </c>
+      <c r="G24" t="s">
+        <v>21</v>
+      </c>
+      <c r="H24" s="4" t="s">
+        <v>37</v>
+      </c>
+    </row>
+    <row r="25" spans="2:8" x14ac:dyDescent="0.45">
+      <c r="B25">
+        <v>3</v>
+      </c>
+      <c r="C25" t="s">
+        <v>25</v>
+      </c>
+      <c r="D25" s="4" t="s">
+        <v>32</v>
+      </c>
+      <c r="F25">
+        <v>3</v>
+      </c>
+      <c r="G25" t="s">
+        <v>20</v>
+      </c>
+      <c r="H25" s="4" t="s">
+        <v>31</v>
+      </c>
+    </row>
+    <row r="26" spans="2:8" ht="28.5" x14ac:dyDescent="0.45">
+      <c r="B26">
+        <v>4</v>
+      </c>
+      <c r="C26" t="s">
+        <v>14</v>
+      </c>
+      <c r="D26" s="3" t="s">
+        <v>40</v>
+      </c>
+      <c r="F26">
+        <v>4</v>
+      </c>
+      <c r="G26" s="2" t="s">
+        <v>7</v>
+      </c>
+      <c r="H26" s="5" t="s">
+        <v>38</v>
+      </c>
+    </row>
+    <row r="27" spans="2:8" ht="28.5" x14ac:dyDescent="0.45">
+      <c r="B27">
+        <v>5</v>
+      </c>
+      <c r="C27" s="2" t="s">
+        <v>6</v>
+      </c>
+      <c r="D27" s="3" t="s">
+        <v>40</v>
+      </c>
+      <c r="F27">
+        <v>5</v>
+      </c>
+      <c r="G27" s="2" t="s">
+        <v>9</v>
+      </c>
+      <c r="H27" s="5" t="s">
+        <v>39</v>
+      </c>
+    </row>
+    <row r="28" spans="2:8" ht="28.5" x14ac:dyDescent="0.45">
+      <c r="B28">
+        <v>6</v>
+      </c>
+      <c r="C28" s="2" t="s">
+        <v>24</v>
+      </c>
+      <c r="D28" s="3" t="s">
+        <v>40</v>
+      </c>
+      <c r="F28">
+        <v>6</v>
+      </c>
+      <c r="G28" s="2" t="s">
+        <v>23</v>
+      </c>
+      <c r="H28" s="3" t="s">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="29" spans="2:8" ht="28.5" x14ac:dyDescent="0.45">
+      <c r="B29">
+        <v>7</v>
+      </c>
+      <c r="C29" s="2" t="s">
+        <v>10</v>
+      </c>
+      <c r="D29" s="3" t="s">
+        <v>40</v>
+      </c>
+      <c r="F29">
+        <v>7</v>
+      </c>
+      <c r="G29" s="2" t="s">
+        <v>26</v>
+      </c>
+      <c r="H29" s="4" t="s">
+        <v>31</v>
+      </c>
+    </row>
+    <row r="30" spans="2:8" x14ac:dyDescent="0.45">
+      <c r="B30">
+        <v>8</v>
+      </c>
+      <c r="C30" s="2" t="s">
+        <v>11</v>
+      </c>
+      <c r="D30" s="3" t="s">
+        <v>40</v>
+      </c>
+      <c r="F30">
+        <v>8</v>
+      </c>
+      <c r="G30" t="s">
+        <v>15</v>
+      </c>
+      <c r="H30" s="3" t="s">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="31" spans="2:8" ht="42.75" x14ac:dyDescent="0.45">
+      <c r="B31">
+        <v>9</v>
+      </c>
+      <c r="C31" s="2" t="s">
+        <v>28</v>
+      </c>
+      <c r="D31" s="5" t="s">
+        <v>33</v>
+      </c>
+      <c r="F31">
+        <v>9</v>
+      </c>
+      <c r="G31" t="s">
+        <v>16</v>
+      </c>
+      <c r="H31" s="4" t="s">
+        <v>31</v>
+      </c>
+    </row>
+    <row r="32" spans="2:8" ht="28.5" x14ac:dyDescent="0.45">
+      <c r="B32">
+        <v>10</v>
+      </c>
+      <c r="C32" s="2" t="s">
+        <v>27</v>
+      </c>
+      <c r="D32" s="3" t="s">
+        <v>40</v>
+      </c>
+      <c r="F32">
+        <v>10</v>
+      </c>
+      <c r="G32" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="H32" s="4" t="s">
+        <v>31</v>
+      </c>
+    </row>
+    <row r="33" spans="2:8" x14ac:dyDescent="0.45">
+      <c r="B33">
+        <v>11</v>
+      </c>
+      <c r="C33" s="2" t="s">
+        <v>18</v>
+      </c>
+      <c r="D33" s="4" t="s">
+        <v>34</v>
+      </c>
+      <c r="F33">
+        <v>11</v>
+      </c>
+      <c r="G33" s="2" t="s">
         <v>17</v>
       </c>
-      <c r="H16" t="s">
-        <v>5</v>
+      <c r="H33" s="4" t="s">
+        <v>31</v>
+      </c>
+    </row>
+    <row r="34" spans="2:8" x14ac:dyDescent="0.45">
+      <c r="B34">
+        <v>11</v>
+      </c>
+      <c r="C34" t="s">
+        <v>22</v>
+      </c>
+      <c r="D34" s="6" t="s">
+        <v>35</v>
       </c>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.78740157499999996" bottom="0.78740157499999996" header="0.3" footer="0.3"/>
-  <tableParts count="2">
+  <tableParts count="4">
     <tablePart r:id="rId1"/>
     <tablePart r:id="rId2"/>
+    <tablePart r:id="rId3"/>
+    <tablePart r:id="rId4"/>
   </tableParts>
 </worksheet>
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
-</file>
-
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement>
-    <_activity xmlns="5f1a80e9-d6bc-4031-b10f-d21f31a30176" xsi:nil="true"/>
-  </documentManagement>
-</p:properties>
-</file>
-
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Dokument" ma:contentTypeID="0x0101005A8D12E036A38A4C82FA7B9385EF06A9" ma:contentTypeVersion="15" ma:contentTypeDescription="Ein neues Dokument erstellen." ma:contentTypeScope="" ma:versionID="5847bb9604bf2beda18d4f7cd4b8a0bc">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns3="5f1a80e9-d6bc-4031-b10f-d21f31a30176" xmlns:ns4="dce9bcdd-9eea-4ca5-a49c-ebeb07b55999" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="02ca0f69bb2fee6ab7e7537675a9b63c" ns3:_="" ns4:_="">
     <xsd:import namespace="5f1a80e9-d6bc-4031-b10f-d21f31a30176"/>
@@ -1063,10 +1399,38 @@
 </ct:contentTypeSchema>
 </file>
 
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement>
+    <_activity xmlns="5f1a80e9-d6bc-4031-b10f-d21f31a30176" xsi:nil="true"/>
+  </documentManagement>
+</p:properties>
+</file>
+
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
+</file>
+
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{C50BBE33-4FF4-4BA4-8155-4BCE83228CBA}">
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{C95935A0-F985-4FFC-9287-686DBD7B5494}">
   <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes"/>
+    <ds:schemaRef ds:uri="http://www.w3.org/2001/XMLSchema"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="5f1a80e9-d6bc-4031-b10f-d21f31a30176"/>
+    <ds:schemaRef ds:uri="dce9bcdd-9eea-4ca5-a49c-ebeb07b55999"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/internal/obd"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
 </file>
@@ -1089,20 +1453,9 @@
 </file>
 
 <file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{C95935A0-F985-4FFC-9287-686DBD7B5494}">
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{C50BBE33-4FF4-4BA4-8155-4BCE83228CBA}">
   <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes"/>
-    <ds:schemaRef ds:uri="http://www.w3.org/2001/XMLSchema"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
-    <ds:schemaRef ds:uri="5f1a80e9-d6bc-4031-b10f-d21f31a30176"/>
-    <ds:schemaRef ds:uri="dce9bcdd-9eea-4ca5-a49c-ebeb07b55999"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/internal/obd"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
 </file>
</xml_diff>